<commit_message>
Add last reference story
</commit_message>
<xml_diff>
--- a/documentation/Agile Stories.xlsx
+++ b/documentation/Agile Stories.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="39">
   <si>
     <t xml:space="preserve">Story #</t>
   </si>
@@ -98,6 +98,12 @@
   </si>
   <si>
     <t xml:space="preserve">Designing a formal langauge defined by a formal grammar and a finite state machine. Implemented the formal language with a data structure that accepts strings considered part of the language.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unity Scene Manager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Creation of a C# class in Unity to load and unload scenes. Scenes are collections of GameObjects and scripts attached to them.</t>
   </si>
   <si>
     <t xml:space="preserve">Used C++ to design and create a UNIX like shell that parses commands and executes tasks based on input. Recognizes basic shell commands and starting/stopping of processes as well as piping.</t>
@@ -424,7 +430,7 @@
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="29.94"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="29.93"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="194.14"/>
   </cols>
   <sheetData>
@@ -603,6 +609,12 @@
       <c r="B13" s="1" t="n">
         <v>5</v>
       </c>
+      <c r="C13" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="n">
@@ -615,7 +627,7 @@
         <v>22</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -626,10 +638,10 @@
         <v>8</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -640,10 +652,10 @@
         <v>8</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -654,10 +666,10 @@
         <v>13</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -668,10 +680,10 @@
         <v>13</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -682,10 +694,10 @@
         <v>13</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Minor formatting and content fixes
</commit_message>
<xml_diff>
--- a/documentation/Agile Stories.xlsx
+++ b/documentation/Agile Stories.xlsx
@@ -64,7 +64,7 @@
     <t xml:space="preserve">Implemented code to do static analysis of programs in LLVM intermediate representation. The project broke down code into basic executable blocks and analyzed each to determine if a secret value was leaked.</t>
   </si>
   <si>
-    <t xml:space="preserve">Input Manager</t>
+    <t xml:space="preserve">Personal Unity Project – Input Manager</t>
   </si>
   <si>
     <t xml:space="preserve">Create a system for managing user input (keyboard/mouse/controller) in the Unity game engine, using official libraries/packages. This includes detecting inputs, but not applying any logic after receiving an input.</t>
@@ -82,7 +82,7 @@
     <t xml:space="preserve">Created an AI solver for the DaMert 3D squares puzzle using depth first search with heuristic based decision making.</t>
   </si>
   <si>
-    <t xml:space="preserve">Unity Save System</t>
+    <t xml:space="preserve">Personal Unity Project – Unity Save System</t>
   </si>
   <si>
     <t xml:space="preserve">Implementation of saving and retrieving objects to and from files in the Unity game engine. This includes defining the object’s fields, collecting data into the fields, and saving it (and going in reverse, too).</t>
@@ -100,7 +100,7 @@
     <t xml:space="preserve">Designing a formal langauge defined by a formal grammar and a finite state machine. Implemented the formal language with a data structure that accepts strings considered part of the language.</t>
   </si>
   <si>
-    <t xml:space="preserve">Unity Scene Manager</t>
+    <t xml:space="preserve">Personal Unity Project – Unity Scene Manager</t>
   </si>
   <si>
     <t xml:space="preserve">Creation of a C# class in Unity to load and unload scenes. Scenes are collections of GameObjects and scripts attached to them.</t>
@@ -109,7 +109,7 @@
     <t xml:space="preserve">Used C++ to design and create a UNIX like shell that parses commands and executes tasks based on input. Recognizes basic shell commands and starting/stopping of processes as well as piping.</t>
   </si>
   <si>
-    <t xml:space="preserve">Tile-Based Pathfinding Algorithm</t>
+    <t xml:space="preserve">Personal Unity Project – Tile-Based Pathfinding Algorithm</t>
   </si>
   <si>
     <t xml:space="preserve">Implement movement across tiles using the A* path finding algorithm, accounting for the possibility that different tiles might have different “movement costs.”</t>
@@ -429,8 +429,8 @@
   <dimension ref="A1:D19"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="29.93"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="50.17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="194.14"/>
   </cols>
   <sheetData>

</xml_diff>